<commit_message>
Align validation demos and prompts across inference console and R8000
</commit_message>
<xml_diff>
--- a/artifacts/pika_20261020_pairing/prompt与人类示教配对.xlsx
+++ b/artifacts/pika_20261020_pairing/prompt与人类示教配对.xlsx
@@ -10991,7 +10991,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>First, place the orange toy tangerine into the light-purple plate. Next, place the brown toy potato into the white storage basket. Finally, place the black computer mouse into the dark-brown wooden tray. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the orange toy tangerine into the dark-brown wooden tray. Next, place the brown toy potato into the light-purple plate. Finally, place the black computer mouse into the white storage basket. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -11001,7 +11001,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -11132,7 +11132,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>First, place the black computer mouse into the dark-brown wooden tray. Next, place the light-green pepper-shaped toy into the light-purple plate. Finally, place the brown toy potato into the white storage basket. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the black computer mouse into the dark-brown wooden tray. Next, place the brown toy potato into the white storage basket. Finally, place the light-green pepper-shaped toy into the light-purple plate. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>First, place the green leaf-shaped toy into the white storage basket. Next, place the orange toy tangerine into the light-purple plate. Finally, place the dark-gray cylindrical cup into the dark-brown wooden tray. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the green leaf-shaped toy into the white storage basket. Next, place the orange toy tangerine into the light-purple plate. Finally, place the brown toy potato into the dark-brown wooden tray. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>First, place the dark-gray cylindrical cup into the dark-brown wooden tray. Next, place the green leaf-shaped toy into the white storage basket. Finally, place the orange toy tangerine into the light-purple plate. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the brown toy potato into the dark-brown wooden tray. Next, place the orange toy tangerine into the light-purple plate. Finally, place the green leaf-shaped toy into the white storage basket. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -11236,7 +11236,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>First, place the orange toy tangerine into the light-purple plate. Next, place the black computer mouse into the dark-brown wooden tray. Finally, place the brown toy potato into the white storage basket. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the orange toy tangerine into the light-purple plate. Next, place the brown toy potato into the white storage basket. Finally, place the black computer mouse into the dark-brown wooden tray. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -11283,7 +11283,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>First, place the brown toy potato into the white storage basket. Next, place the black computer mouse into the dark-brown wooden tray. Finally, place the orange toy tangerine into the light-purple plate. Complete all three placements in this order without moving unrelated objects.</t>
+          <t>First, place the black computer mouse into the dark-brown wooden tray. Next, place the brown toy potato into the white storage basket. Finally, place the orange toy tangerine into the light-purple plate. Complete all three placements in this order without moving unrelated objects.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>candidate_recording_order_needs_separate_confirmation</t>
+          <t>visually_reviewed_20261022</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">

</xml_diff>